<commit_message>
Séparation query chroma en query documentation et query mails
</commit_message>
<xml_diff>
--- a/fastapi-backend/data/Planning général_màj au 20260604.xlsx
+++ b/fastapi-backend/data/Planning général_màj au 20260604.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Windows\Documents\000_mystuff\0_llm-rag\wip\fastapi-backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F8D35DB-6CDA-415F-B93E-EE34EBDCE24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED60105-AC16-4057-9438-B800AA49288D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>Réalisation des places définitives en Z1</t>
   </si>
@@ -136,6 +136,15 @@
   </si>
   <si>
     <t>Fin</t>
+  </si>
+  <si>
+    <t>Lot 6</t>
+  </si>
+  <si>
+    <t>CB</t>
+  </si>
+  <si>
+    <t>Intervenant</t>
   </si>
 </sst>
 </file>
@@ -145,10 +154,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -459,216 +474,244 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="34.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" style="1" customWidth="1"/>
-    <col min="6" max="6" width="36.33203125" customWidth="1"/>
+    <col min="3" max="3" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30" style="1" customWidth="1"/>
+    <col min="7" max="7" width="36.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>31</v>
       </c>
       <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>